<commit_message>
erz-rts: обновление 2026-07-13 12:18 UTC
</commit_message>
<xml_diff>
--- a/erz-rts-leadgen/erz_rts.xlsx
+++ b/erz-rts-leadgen/erz_rts.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="РТС-тендер" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ЕРЗ.РФ (застройщики)'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ЕРЗ.РФ (застройщики)'!$A$1:$O$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'РТС-тендер'!$A$1:$N$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -59,10 +63,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,22 +439,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,52 +482,1444 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Регион</t>
+          <t>Рейтинг РФ</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Регион (вид рейтинга)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Доля в регионе</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Строится в регионе</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Всего проектов в ЕРЗ</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Год основания</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Руководитель</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Осн. ОКВЭД</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Объект строительства</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Стадия</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Срок сдачи</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Адрес</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Ссылка</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ПИК</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "ПИК СЗ"</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>7713011336</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>№2 в РФ</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>13.43%</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2 239 980 м²</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Бондарев Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>64.99.3</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Баррикадная, д 19 стр 1</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/pik-429726001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=429726001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>ГК Самолет</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "ГК "САМОЛЕТ"</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>9731004688</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>№1 в РФ</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Московская обл</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>6.48%</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>1 079 976 м²</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Акиньшина Анна Николаевна</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Московская обл, г Красногорск, ул Липовой Рощи, д 1 к 3, помещ 18, ком 3</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-samolet-2366201001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=2366201001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>MR Group</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МР ГРУПП"</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>3906412859</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>№12 в РФ</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Калининградская обл</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>6.31%</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>1 051 717 м²</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Рыхлицкая Анастасия Владимировна</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>46.73</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>238434, КАЛИНИНГРАДСКАЯ ОБЛАСТЬ, М.О. ГУРЬЕВСКИЙ, П. ЛЕСНОЕ, УЛ. АВТОДОРОЖНАЯ, СТР. 3, ОФИС 2</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/mr-group-430836001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=430836001</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ДОНСТРОЙ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>АО "ДОНСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>6154012871</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>№19 в РФ</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Ростовская обл</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>4.78%</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>797 384 м²</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Мардахаев Максим Биняминович</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>41.20.1</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Ростовская обл, г Таганрог, ул Поляковское Шоссе, д 16А</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/donstroj-430278001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=430278001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ГК ФСК</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ФСК"</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>7708332091</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>№5 в РФ</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>4.45%</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>741 325 м²</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Трубников Дмитрий Александрович</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>64.99</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Каланчевская, д 32, помещ 4/2П</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-fsk-755344001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=755344001</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Level Group</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ООО "А-ЛЕВЕЛ ГРУПП"</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>9701095007</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>№21 в РФ</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Московская обл</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>3.63%</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>605 520 м²</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Валиев Хуршид Абдуманноп Угли</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>46.72</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Московская обл, г Химки, ул Жуковского, д 10, помещ 29А</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/level-group-6150430001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=6150430001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ГК А101</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ГК 101 А</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>4401021566</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>№22 в РФ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Костромская обл</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>3.58%</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>597 205 м²</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Парфенцев Алексей Сергеевич</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>52.21.24</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>г Кострома, ул Смирнова Юрия, д 30А, офис 74</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-a101-1075233001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=1075233001</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ГК АБСОЛЮТ</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК "АБСОЛЮТ"</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>0264064744</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>№27 в РФ</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Респ Башкортостан</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2.71%</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>451 633 м²</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Мифтахов Артур Рашатович</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>45.11.2</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Респ Башкортостан, г Нефтекамск, ул Янаульская, д 1А</t>
+        </is>
+      </c>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-absoljut-934095001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=934095001</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ГК Страна Девелопмент</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>№10 в РФ</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>moskva</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2.45%</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>408 286 м²</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-strana-development-5339663001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=5339663001</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ГК ОСНОВА</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>АО "ГК "ОСНОВА"</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>9715264590</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>№36 в РФ</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Московская обл</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2.22%</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>369 553 м²</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Попов Евгений Владимирович</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Московская обл, г Видное, Белокаменное шоссе, д 20</t>
+        </is>
+      </c>
+      <c r="O11" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-osnova-6201034001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=6201034001</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Брусника</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ООО "БКП"</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>6671139146</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>№8 в РФ</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Свердловская обл</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2.09%</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>348 043 м²</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "БРУСНИКА. СТРОИТЕЛЬСТВО И ДЕВЕЛОПМЕНТ"</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>41.20.9</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>г Екатеринбург, ул Гоголя, стр 18, помещ 329</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/brusnika-733498001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=733498001</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Группа ЛСР</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ПАО "ГРУППА ЛСР"</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>7838360491</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>№11 в РФ</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>г Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2.06%</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>342 826 м²</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Кутузов Дмитрий Владимирович</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>64.20</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>190031, Г.САНКТ-ПЕТЕРБУРГ, УЛ. КАЗАНСКАЯ, Д.36ЛИТЕРБ, ЭТАЖ 4 ПОМ 32-Н (18) КАБ 404</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-lsr-429468001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=429468001</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ГК Гранель</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ООО "ГК ГРАНЕЛЬ"</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>1655486295</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>№16 в РФ</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Респ Татарстан</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>1.86%</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>310 101 м²</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "РАЛЕН"</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>46.90</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>г Казань, ул Миславского, д 9Б, офис 320</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-granel-955386001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=955386001</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Фонд реновации</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>ФОНД РЕНОВАЦИИ</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>7703434808</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>№57 в РФ</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>1.68%</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>280 348 м²</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>319</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Степанов Максим Сергеевич</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>71.12.2</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Ильинка, д 13</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/moskovskij-fond-renovacii-zhiloj-zastrojki-14543898001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=14543898001</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ГК Главстрой</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ООО ГК "ГЛАВСТРОЙ"</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>6671047270</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>№64 в РФ</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Свердловская обл</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>1.6%</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>266 873 м²</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Губаев Камиль Фаилович</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>41.20</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>620043, СВЕРДЛОВСКАЯ ОБЛАСТЬ, Г. ЕКАТЕРИНБУРГ, УЛ. РЕПИНА, СТР. 42А, ОФИС 202</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-kompanij-glavstroj-1961151001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=1961151001</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Группа Аквилон</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>ООО "АКВИЛОН ГРУППА КОМПАНИЙ"</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2312136434</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>№18 в РФ</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Краснодарский край</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>1.52%</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>253 658 м²</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Лебедева Олеся Валерьевна</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>47.54</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>г Краснодар, ул Сормовская, д 7 литера г, помещ 87/88</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-akvilon-391375001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=391375001</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Группа Эталон</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>АО "ГК "ЭТАЛОН"</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>7814116230</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>№13 в РФ</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>1.48%</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>246 967 м²</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>1987</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Бородин Юрий Алексеевич</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>70.10</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Новоалексеевская, д 16 стр 5</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/gruppa-etalon-1331499001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=1331499001</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13 12:18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Мангазея</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>ООО "МАНГАЗЕЯ"</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>7704808608</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>№93 в РФ</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>г Москва</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>1.19%</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>199 002 м²</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Янчуков Сергей Валентинович</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>70.22</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>г Москва, ул Автозаводская, д 2, помещ 5/1П</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>https://erzrf.ru/zastroyschiki/brand/mangazeja-3126628001?region=moskva&amp;regionKey=143443001&amp;costType=1&amp;organizationId=3126628001</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M2"/>
+  <autoFilter ref="A1:O19"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId18"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>